<commit_message>
pdf + resumo + horas extra
</commit_message>
<xml_diff>
--- a/relatorio.xlsx
+++ b/relatorio.xlsx
@@ -4,20 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="Relatorio Ponto" state="visible" r:id="rId4"/>
+    <sheet sheetId="1" name="Relatório Ponto" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
-  <si>
-    <t>ID Registo</t>
-  </si>
-  <si>
-    <t>Funcionário ID</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Funcionário</t>
   </si>
@@ -415,19 +409,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="24" customWidth="1"/>
-    <col min="4" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="22" customWidth="1"/>
-    <col min="7" max="8" width="14" customWidth="1"/>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="6" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -445,12 +437,6 @@
       </c>
       <c r="F1" s="1" t="s">
         <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>